<commit_message>
docs(deliverables): refresh notebook, workbook and write-ups for the retrain
Re-execute the pipeline notebook (and its package copies), update the
Excel workbook cells and priority rows, and replace MAE 5.859 -> 5.862,
improvement 2.2% -> 2.1% and R2 0.070 -> 0.069 in the READMEs,
methodology and video script. Refresh stale package images 01 and 07-09.
</commit_message>
<xml_diff>
--- a/dist/dashboard_package/Dashboard.xlsx
+++ b/dist/dashboard_package/Dashboard.xlsx
@@ -18,7 +18,7 @@
     <sheet name="History_Data" sheetId="3" r:id="rId3"/>
     <sheet name="Model_Check" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -104,7 +104,7 @@
     <t>Model check</t>
   </si>
   <si>
-    <t>Gradient boosting MAE 5.86 pp/yr vs baseline 5.99 pp/yr (+2.2%). R² 0.070. NOAA heat is context only. Use the model to rank field checks, not as proof of tourism causality.</t>
+    <t>Gradient boosting MAE 5.86 pp/yr vs baseline 5.99 pp/yr (+2.1%). R² 0.069. NOAA heat is context only. Use the model to rank field checks, not as proof of tourism causality.</t>
   </si>
   <si>
     <t>Rank</t>
@@ -1911,15 +1911,15 @@
       </c>
       <c r="I40" s="7">
         <f>Model_Check!B4</f>
-        <v>5.859</v>
+        <v>5.862</v>
       </c>
       <c r="J40" s="7">
         <f>Model_Check!C4</f>
-        <v>7.7389999999999999</v>
+        <v>7.741</v>
       </c>
       <c r="K40" s="7">
         <f>Model_Check!D4</f>
-        <v>7.0000000000000007E-2</v>
+        <v>0.069</v>
       </c>
     </row>
     <row r="41" spans="1:13" ht="30" customHeight="1">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="J41" s="7">
         <f>Model_Check!C5</f>
-        <v>8.0169999999999995</v>
+        <v>8.016</v>
       </c>
       <c r="K41" s="7">
         <f>Model_Check!D5</f>
@@ -3624,91 +3624,91 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="27.6">
+    <row r="37" spans="1:13">
       <c r="A37" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B37">
         <v>36</v>
       </c>
       <c r="C37" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="D37" s="5">
-        <v>22.55</v>
+        <v>48.02</v>
       </c>
       <c r="E37" s="5">
-        <v>-10.29</v>
+        <v>-11.25</v>
       </c>
       <c r="F37" s="5">
-        <v>4.04</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="G37" s="5">
-        <v>-0.14582637801605128</v>
+        <v>-0.6145464227998586</v>
       </c>
       <c r="H37" s="5">
-        <v>-16.400211854119814</v>
+        <v>-16.86893189890362</v>
       </c>
       <c r="I37" s="5">
-        <v>13.51619058131379</v>
+        <v>13.047470536529982</v>
       </c>
       <c r="J37" t="s">
         <v>58</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="M37" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" ht="27.6">
       <c r="A38" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B38">
         <v>37</v>
       </c>
       <c r="C38" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="D38" s="5">
-        <v>48.02</v>
+        <v>22.55</v>
       </c>
       <c r="E38" s="5">
-        <v>-11.25</v>
+        <v>-10.29</v>
       </c>
       <c r="F38" s="5">
-        <v>2.0499999999999998</v>
+        <v>4.04</v>
       </c>
       <c r="G38" s="5">
-        <v>0.59140515831126883</v>
+        <v>-0.14582637801605147</v>
       </c>
       <c r="H38" s="5">
-        <v>-15.662980317792496</v>
+        <v>-16.400211854119814</v>
       </c>
       <c r="I38" s="5">
-        <v>14.25342211764111</v>
+        <v>13.516190581313788</v>
       </c>
       <c r="J38" t="s">
         <v>58</v>
       </c>
       <c r="K38" s="6" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="M38" s="6" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:13" ht="27.6">
       <c r="A39" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B39">
         <v>38</v>
@@ -3717,22 +3717,22 @@
         <v>56</v>
       </c>
       <c r="D39" s="5">
-        <v>14.69</v>
+        <v>26.56</v>
       </c>
       <c r="E39" s="5">
-        <v>-5.81</v>
+        <v>4.2699999999999996</v>
       </c>
       <c r="F39" s="5">
         <v>4.04</v>
       </c>
       <c r="G39" s="5">
-        <v>0.77009129264920617</v>
+        <v>-0.03075295618797179</v>
       </c>
       <c r="H39" s="5">
-        <v>-15.484294183454557</v>
+        <v>-16.285138432291735</v>
       </c>
       <c r="I39" s="5">
-        <v>14.432108251979049</v>
+        <v>13.631264003141869</v>
       </c>
       <c r="J39" t="s">
         <v>58</v>
@@ -3744,12 +3744,12 @@
         <v>35</v>
       </c>
       <c r="M39" s="6" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="40" spans="1:13" ht="27.6">
       <c r="A40" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B40">
         <v>39</v>
@@ -3758,22 +3758,22 @@
         <v>56</v>
       </c>
       <c r="D40" s="5">
-        <v>26.56</v>
+        <v>14.69</v>
       </c>
       <c r="E40" s="5">
-        <v>4.2699999999999996</v>
+        <v>-5.81</v>
       </c>
       <c r="F40" s="5">
         <v>4.04</v>
       </c>
       <c r="G40" s="5">
-        <v>1.1751986249231563</v>
+        <v>0.770091292649206</v>
       </c>
       <c r="H40" s="5">
-        <v>-15.079186851180607</v>
+        <v>-15.484294183454558</v>
       </c>
       <c r="I40" s="5">
-        <v>14.837215584252998</v>
+        <v>14.432108251979045</v>
       </c>
       <c r="J40" t="s">
         <v>58</v>
@@ -3785,7 +3785,7 @@
         <v>35</v>
       </c>
       <c r="M40" s="6" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="41" spans="1:13">
@@ -13138,19 +13138,19 @@
         <v>121</v>
       </c>
       <c r="B4" s="7">
-        <v>5.859</v>
+        <v>5.862</v>
       </c>
       <c r="C4" s="7">
-        <v>7.7389999999999999</v>
+        <v>7.741</v>
       </c>
       <c r="D4" s="7">
-        <v>7.0000000000000007E-2</v>
+        <v>0.069</v>
       </c>
       <c r="F4" t="s">
         <v>122</v>
       </c>
       <c r="G4" s="8">
-        <v>2.1965089167881494E-2</v>
+        <v>2.1488199341510157E-2</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -13161,7 +13161,7 @@
         <v>6.0739999999999998</v>
       </c>
       <c r="C5" s="7">
-        <v>8.0169999999999995</v>
+        <v>8.016</v>
       </c>
       <c r="D5" s="7">
         <v>2E-3</v>

</xml_diff>